<commit_message>
Refactor CLM training functions and remove unused code
</commit_message>
<xml_diff>
--- a/valid_unique_smiles_28_02_2025.xlsx
+++ b/valid_unique_smiles_28_02_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Computer\Meh!!!!!!!\workspace\VIT_LAB\SingletFission_ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AB1588-414F-44D8-9BA5-9E4E59770F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2A18FD-5918-42F1-9BD0-40B5E5F8777A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="889" xr2:uid="{9748B68E-534E-4D07-B84B-E3A578C6F34D}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="889" firstSheet="2" activeTab="4" xr2:uid="{9748B68E-534E-4D07-B84B-E3A578C6F34D}"/>
   </bookViews>
   <sheets>
     <sheet name="valid_unique_smiles_28_02_2025" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="Benzene c1ccccc348" sheetId="3" r:id="rId11"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Polar grp  N+ ( O- )'!$A$1:$C$408</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">valid_unique_smiles_28_02_2025!$A$1:$C$2879</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -53810,10 +53811,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2081DE18-20BE-4B1B-93EE-F628AB19DCC6}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:C408"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="50.6640625" customWidth="1"/>
+    <col min="2" max="2" width="63.44140625" customWidth="1"/>
     <col min="3" max="3" width="78.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -53828,7 +53830,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -53839,7 +53841,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -53850,7 +53852,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -53861,7 +53863,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>27</v>
       </c>
@@ -53872,7 +53874,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>39</v>
       </c>
@@ -53883,7 +53885,7 @@
         <v>6208</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>59</v>
       </c>
@@ -53905,7 +53907,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>93</v>
       </c>
@@ -53916,7 +53918,7 @@
         <v>6210</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
@@ -53927,7 +53929,7 @@
         <v>6211</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>103</v>
       </c>
@@ -53949,7 +53951,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>167</v>
       </c>
@@ -53960,7 +53962,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>175</v>
       </c>
@@ -53971,7 +53973,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>205</v>
       </c>
@@ -53982,7 +53984,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>217</v>
       </c>
@@ -53993,7 +53995,7 @@
         <v>6214</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>267</v>
       </c>
@@ -54004,7 +54006,7 @@
         <v>6215</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>273</v>
       </c>
@@ -54015,7 +54017,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>289</v>
       </c>
@@ -54037,7 +54039,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>319</v>
       </c>
@@ -54070,7 +54072,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>367</v>
       </c>
@@ -54103,7 +54105,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>401</v>
       </c>
@@ -54114,7 +54116,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>409</v>
       </c>
@@ -54136,7 +54138,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>429</v>
       </c>
@@ -54147,7 +54149,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>431</v>
       </c>
@@ -54158,7 +54160,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>433</v>
       </c>
@@ -54169,7 +54171,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>447</v>
       </c>
@@ -54180,7 +54182,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>475</v>
       </c>
@@ -54191,7 +54193,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>477</v>
       </c>
@@ -54202,7 +54204,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>495</v>
       </c>
@@ -54213,7 +54215,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>501</v>
       </c>
@@ -54224,7 +54226,7 @@
         <v>6217</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>549</v>
       </c>
@@ -54257,7 +54259,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>601</v>
       </c>
@@ -54279,7 +54281,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>629</v>
       </c>
@@ -54301,7 +54303,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>645</v>
       </c>
@@ -54323,7 +54325,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>683</v>
       </c>
@@ -54334,7 +54336,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>691</v>
       </c>
@@ -54345,7 +54347,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>707</v>
       </c>
@@ -54356,7 +54358,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>709</v>
       </c>
@@ -54378,7 +54380,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>721</v>
       </c>
@@ -54389,7 +54391,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>723</v>
       </c>
@@ -54411,7 +54413,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>751</v>
       </c>
@@ -54422,7 +54424,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>773</v>
       </c>
@@ -54433,7 +54435,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>797</v>
       </c>
@@ -54444,7 +54446,7 @@
         <v>6219</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>829</v>
       </c>
@@ -54466,7 +54468,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>863</v>
       </c>
@@ -54477,7 +54479,7 @@
         <v>6210</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>873</v>
       </c>
@@ -54488,7 +54490,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>905</v>
       </c>
@@ -54499,7 +54501,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>911</v>
       </c>
@@ -54510,7 +54512,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>915</v>
       </c>
@@ -54532,7 +54534,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>927</v>
       </c>
@@ -54543,7 +54545,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>939</v>
       </c>
@@ -54554,7 +54556,7 @@
         <v>6221</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>951</v>
       </c>
@@ -54576,7 +54578,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>957</v>
       </c>
@@ -54598,7 +54600,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>1021</v>
       </c>
@@ -54609,7 +54611,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>1029</v>
       </c>
@@ -54620,7 +54622,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>1047</v>
       </c>
@@ -54631,7 +54633,7 @@
         <v>6208</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>1065</v>
       </c>
@@ -54642,7 +54644,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>1089</v>
       </c>
@@ -54653,7 +54655,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>1091</v>
       </c>
@@ -54664,7 +54666,7 @@
         <v>6193</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>1121</v>
       </c>
@@ -54675,7 +54677,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>1157</v>
       </c>
@@ -54686,7 +54688,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>1161</v>
       </c>
@@ -54697,7 +54699,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>1181</v>
       </c>
@@ -54708,7 +54710,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>1185</v>
       </c>
@@ -54752,7 +54754,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>1223</v>
       </c>
@@ -54763,7 +54765,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>1231</v>
       </c>
@@ -54774,7 +54776,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>1237</v>
       </c>
@@ -54785,7 +54787,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>1337</v>
       </c>
@@ -54796,7 +54798,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>1341</v>
       </c>
@@ -54829,7 +54831,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>1429</v>
       </c>
@@ -54851,7 +54853,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>1445</v>
       </c>
@@ -54862,7 +54864,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>1473</v>
       </c>
@@ -54873,7 +54875,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>1483</v>
       </c>
@@ -54884,7 +54886,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>1495</v>
       </c>
@@ -54895,7 +54897,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>1537</v>
       </c>
@@ -54906,7 +54908,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>1541</v>
       </c>
@@ -54917,7 +54919,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>1555</v>
       </c>
@@ -54928,7 +54930,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>1587</v>
       </c>
@@ -54939,7 +54941,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>1595</v>
       </c>
@@ -54950,7 +54952,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>1599</v>
       </c>
@@ -54961,7 +54963,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>1629</v>
       </c>
@@ -54972,7 +54974,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>1643</v>
       </c>
@@ -54994,7 +54996,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>1653</v>
       </c>
@@ -55005,7 +55007,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>1655</v>
       </c>
@@ -55038,7 +55040,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>1671</v>
       </c>
@@ -55049,7 +55051,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>1673</v>
       </c>
@@ -55060,7 +55062,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>1691</v>
       </c>
@@ -55071,7 +55073,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>1735</v>
       </c>
@@ -55082,7 +55084,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>1739</v>
       </c>
@@ -55093,7 +55095,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>1759</v>
       </c>
@@ -55104,7 +55106,7 @@
         <v>6211</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>1779</v>
       </c>
@@ -55126,7 +55128,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>1801</v>
       </c>
@@ -55148,7 +55150,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>1823</v>
       </c>
@@ -55159,7 +55161,7 @@
         <v>6222</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>1847</v>
       </c>
@@ -55170,7 +55172,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>1855</v>
       </c>
@@ -55181,7 +55183,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>1861</v>
       </c>
@@ -55192,7 +55194,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>1867</v>
       </c>
@@ -55214,7 +55216,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>1875</v>
       </c>
@@ -55225,7 +55227,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>1877</v>
       </c>
@@ -55236,7 +55238,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>1879</v>
       </c>
@@ -55247,7 +55249,7 @@
         <v>6211</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>1885</v>
       </c>
@@ -55291,7 +55293,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>1923</v>
       </c>
@@ -55302,7 +55304,7 @@
         <v>6225</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>1941</v>
       </c>
@@ -55346,7 +55348,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>1977</v>
       </c>
@@ -55368,7 +55370,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>2035</v>
       </c>
@@ -55379,7 +55381,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>2041</v>
       </c>
@@ -55390,7 +55392,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>2053</v>
       </c>
@@ -55401,7 +55403,7 @@
         <v>6227</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>2055</v>
       </c>
@@ -55412,7 +55414,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>2061</v>
       </c>
@@ -55423,7 +55425,7 @@
         <v>6228</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>2067</v>
       </c>
@@ -55434,7 +55436,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>2075</v>
       </c>
@@ -55456,7 +55458,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>2083</v>
       </c>
@@ -55467,7 +55469,7 @@
         <v>6229</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>2091</v>
       </c>
@@ -55489,7 +55491,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>2129</v>
       </c>
@@ -55500,7 +55502,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>2145</v>
       </c>
@@ -55511,7 +55513,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>2147</v>
       </c>
@@ -55533,7 +55535,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>2165</v>
       </c>
@@ -55555,7 +55557,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>2185</v>
       </c>
@@ -55577,7 +55579,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>2199</v>
       </c>
@@ -55588,7 +55590,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>2201</v>
       </c>
@@ -55599,7 +55601,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>2203</v>
       </c>
@@ -55621,7 +55623,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>2215</v>
       </c>
@@ -55632,7 +55634,7 @@
         <v>6226</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>2223</v>
       </c>
@@ -55643,7 +55645,7 @@
         <v>6221</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>2243</v>
       </c>
@@ -55654,7 +55656,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>2259</v>
       </c>
@@ -55687,7 +55689,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>2277</v>
       </c>
@@ -55698,7 +55700,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>2321</v>
       </c>
@@ -55709,7 +55711,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>2335</v>
       </c>
@@ -55720,7 +55722,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
         <v>2351</v>
       </c>
@@ -55742,7 +55744,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>2377</v>
       </c>
@@ -55753,7 +55755,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>2391</v>
       </c>
@@ -55764,7 +55766,7 @@
         <v>6230</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>2413</v>
       </c>
@@ -55775,7 +55777,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>2443</v>
       </c>
@@ -55786,7 +55788,7 @@
         <v>6231</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>2457</v>
       </c>
@@ -55797,7 +55799,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
         <v>2487</v>
       </c>
@@ -55830,7 +55832,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>2563</v>
       </c>
@@ -55841,7 +55843,7 @@
         <v>6229</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
         <v>2565</v>
       </c>
@@ -55852,7 +55854,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>2567</v>
       </c>
@@ -55863,7 +55865,7 @@
         <v>6229</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>2573</v>
       </c>
@@ -55874,7 +55876,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>2583</v>
       </c>
@@ -55885,7 +55887,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>2645</v>
       </c>
@@ -55896,7 +55898,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>2653</v>
       </c>
@@ -55918,7 +55920,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>2661</v>
       </c>
@@ -55929,7 +55931,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>2679</v>
       </c>
@@ -55962,7 +55964,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="1" t="s">
         <v>2739</v>
       </c>
@@ -55973,7 +55975,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>2795</v>
       </c>
@@ -56017,7 +56019,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
         <v>2871</v>
       </c>
@@ -56028,7 +56030,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="1" t="s">
         <v>2907</v>
       </c>
@@ -56039,7 +56041,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="1" t="s">
         <v>2943</v>
       </c>
@@ -56050,7 +56052,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="1" t="s">
         <v>2947</v>
       </c>
@@ -56061,7 +56063,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="1" t="s">
         <v>2953</v>
       </c>
@@ -56094,7 +56096,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="1" t="s">
         <v>3027</v>
       </c>
@@ -56127,7 +56129,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="1" t="s">
         <v>3039</v>
       </c>
@@ -56149,7 +56151,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="1" t="s">
         <v>3061</v>
       </c>
@@ -56160,7 +56162,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="1" t="s">
         <v>3071</v>
       </c>
@@ -56171,7 +56173,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="1" t="s">
         <v>3073</v>
       </c>
@@ -56193,7 +56195,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="1" t="s">
         <v>3133</v>
       </c>
@@ -56215,7 +56217,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" s="1" t="s">
         <v>3149</v>
       </c>
@@ -56237,7 +56239,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" s="1" t="s">
         <v>3231</v>
       </c>
@@ -56248,7 +56250,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="1" t="s">
         <v>3237</v>
       </c>
@@ -56259,7 +56261,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" s="1" t="s">
         <v>3257</v>
       </c>
@@ -56281,7 +56283,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" s="1" t="s">
         <v>3267</v>
       </c>
@@ -56292,7 +56294,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" s="1" t="s">
         <v>3273</v>
       </c>
@@ -56303,7 +56305,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" s="1" t="s">
         <v>3281</v>
       </c>
@@ -56314,7 +56316,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="1" t="s">
         <v>3285</v>
       </c>
@@ -56325,7 +56327,7 @@
         <v>6184</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="1" t="s">
         <v>3287</v>
       </c>
@@ -56336,7 +56338,7 @@
         <v>6211</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="1" t="s">
         <v>3295</v>
       </c>
@@ -56358,7 +56360,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" s="1" t="s">
         <v>3307</v>
       </c>
@@ -56369,7 +56371,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="1" t="s">
         <v>3323</v>
       </c>
@@ -56380,7 +56382,7 @@
         <v>6222</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="1" t="s">
         <v>3327</v>
       </c>
@@ -56391,7 +56393,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="1" t="s">
         <v>3337</v>
       </c>
@@ -56402,7 +56404,7 @@
         <v>6226</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="1" t="s">
         <v>3339</v>
       </c>
@@ -56413,7 +56415,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" s="1" t="s">
         <v>3351</v>
       </c>
@@ -56424,7 +56426,7 @@
         <v>6233</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="1" t="s">
         <v>3369</v>
       </c>
@@ -56435,7 +56437,7 @@
         <v>6232</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="1" t="s">
         <v>3375</v>
       </c>
@@ -56446,7 +56448,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" s="1" t="s">
         <v>3379</v>
       </c>
@@ -56468,7 +56470,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" s="1" t="s">
         <v>3419</v>
       </c>
@@ -56490,7 +56492,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="1" t="s">
         <v>3453</v>
       </c>
@@ -56512,7 +56514,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" s="1" t="s">
         <v>3473</v>
       </c>
@@ -56534,7 +56536,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" s="1" t="s">
         <v>3501</v>
       </c>
@@ -56545,7 +56547,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" s="1" t="s">
         <v>3513</v>
       </c>
@@ -56556,7 +56558,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" s="1" t="s">
         <v>3515</v>
       </c>
@@ -56567,7 +56569,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" s="1" t="s">
         <v>3541</v>
       </c>
@@ -56600,7 +56602,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" s="1" t="s">
         <v>3567</v>
       </c>
@@ -56611,7 +56613,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" s="1" t="s">
         <v>3585</v>
       </c>
@@ -56622,7 +56624,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" s="1" t="s">
         <v>3603</v>
       </c>
@@ -56633,7 +56635,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="1" t="s">
         <v>3641</v>
       </c>
@@ -56655,7 +56657,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" s="1" t="s">
         <v>3655</v>
       </c>
@@ -56666,7 +56668,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" s="1" t="s">
         <v>3701</v>
       </c>
@@ -56688,7 +56690,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" s="1" t="s">
         <v>3731</v>
       </c>
@@ -56721,7 +56723,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" s="1" t="s">
         <v>3787</v>
       </c>
@@ -56754,7 +56756,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="1" t="s">
         <v>3873</v>
       </c>
@@ -56787,7 +56789,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="1" t="s">
         <v>3923</v>
       </c>
@@ -56798,7 +56800,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="1" t="s">
         <v>3927</v>
       </c>
@@ -56809,7 +56811,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="1" t="s">
         <v>3931</v>
       </c>
@@ -56820,7 +56822,7 @@
         <v>6221</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="1" t="s">
         <v>3935</v>
       </c>
@@ -56842,7 +56844,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" s="1" t="s">
         <v>3951</v>
       </c>
@@ -56864,7 +56866,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="1" t="s">
         <v>3959</v>
       </c>
@@ -56875,7 +56877,7 @@
         <v>6234</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" s="1" t="s">
         <v>3963</v>
       </c>
@@ -56897,7 +56899,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" s="1" t="s">
         <v>4029</v>
       </c>
@@ -56908,7 +56910,7 @@
         <v>6210</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" s="1" t="s">
         <v>4059</v>
       </c>
@@ -56930,7 +56932,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" s="1" t="s">
         <v>4089</v>
       </c>
@@ -56941,7 +56943,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" s="1" t="s">
         <v>4095</v>
       </c>
@@ -56952,7 +56954,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" s="1" t="s">
         <v>4103</v>
       </c>
@@ -56963,7 +56965,7 @@
         <v>6226</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" s="1" t="s">
         <v>4111</v>
       </c>
@@ -56974,7 +56976,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" s="1" t="s">
         <v>4115</v>
       </c>
@@ -56985,7 +56987,7 @@
         <v>6225</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" s="1" t="s">
         <v>4131</v>
       </c>
@@ -56996,7 +56998,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" s="1" t="s">
         <v>4139</v>
       </c>
@@ -57007,7 +57009,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A291" s="1" t="s">
         <v>4141</v>
       </c>
@@ -57018,7 +57020,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A292" s="1" t="s">
         <v>4151</v>
       </c>
@@ -57040,7 +57042,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" s="1" t="s">
         <v>4159</v>
       </c>
@@ -57051,7 +57053,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" s="1" t="s">
         <v>4163</v>
       </c>
@@ -57062,7 +57064,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" s="1" t="s">
         <v>4167</v>
       </c>
@@ -57084,7 +57086,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" s="1" t="s">
         <v>4191</v>
       </c>
@@ -57106,7 +57108,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A300" s="1" t="s">
         <v>4213</v>
       </c>
@@ -57117,7 +57119,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" s="1" t="s">
         <v>4287</v>
       </c>
@@ -57128,7 +57130,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" s="1" t="s">
         <v>4289</v>
       </c>
@@ -57150,7 +57152,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" s="1" t="s">
         <v>4333</v>
       </c>
@@ -57161,7 +57163,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A305" s="1" t="s">
         <v>4335</v>
       </c>
@@ -57172,7 +57174,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A306" s="1" t="s">
         <v>4357</v>
       </c>
@@ -57183,7 +57185,7 @@
         <v>6229</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A307" s="1" t="s">
         <v>4363</v>
       </c>
@@ -57194,7 +57196,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A308" s="1" t="s">
         <v>4373</v>
       </c>
@@ -57227,7 +57229,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A311" s="1" t="s">
         <v>4425</v>
       </c>
@@ -57238,7 +57240,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" s="1" t="s">
         <v>4447</v>
       </c>
@@ -57249,7 +57251,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A313" s="1" t="s">
         <v>4453</v>
       </c>
@@ -57260,7 +57262,7 @@
         <v>6236</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A314" s="1" t="s">
         <v>4469</v>
       </c>
@@ -57271,7 +57273,7 @@
         <v>6221</v>
       </c>
     </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A315" s="1" t="s">
         <v>4475</v>
       </c>
@@ -57282,7 +57284,7 @@
         <v>6218</v>
       </c>
     </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" s="1" t="s">
         <v>4479</v>
       </c>
@@ -57293,7 +57295,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" s="1" t="s">
         <v>4481</v>
       </c>
@@ -57304,7 +57306,7 @@
         <v>6210</v>
       </c>
     </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" s="1" t="s">
         <v>4517</v>
       </c>
@@ -57315,7 +57317,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" s="1" t="s">
         <v>4525</v>
       </c>
@@ -57326,7 +57328,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" s="1" t="s">
         <v>4557</v>
       </c>
@@ -57348,7 +57350,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" s="1" t="s">
         <v>4603</v>
       </c>
@@ -57359,7 +57361,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" s="1" t="s">
         <v>4607</v>
       </c>
@@ -57370,7 +57372,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A324" s="1" t="s">
         <v>4617</v>
       </c>
@@ -57392,7 +57394,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A326" s="1" t="s">
         <v>4653</v>
       </c>
@@ -57403,7 +57405,7 @@
         <v>6228</v>
       </c>
     </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" s="1" t="s">
         <v>4673</v>
       </c>
@@ -57414,7 +57416,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" s="1" t="s">
         <v>4677</v>
       </c>
@@ -57436,7 +57438,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="330" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" s="1" t="s">
         <v>4693</v>
       </c>
@@ -57447,7 +57449,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="331" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" s="1" t="s">
         <v>4729</v>
       </c>
@@ -57458,7 +57460,7 @@
         <v>6211</v>
       </c>
     </row>
-    <row r="332" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A332" s="1" t="s">
         <v>4739</v>
       </c>
@@ -57469,7 +57471,7 @@
         <v>6232</v>
       </c>
     </row>
-    <row r="333" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" s="1" t="s">
         <v>4767</v>
       </c>
@@ -57491,7 +57493,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="335" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" s="1" t="s">
         <v>4795</v>
       </c>
@@ -57502,7 +57504,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A336" s="1" t="s">
         <v>4797</v>
       </c>
@@ -57524,7 +57526,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A338" s="1" t="s">
         <v>4809</v>
       </c>
@@ -57535,7 +57537,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" s="1" t="s">
         <v>4861</v>
       </c>
@@ -57546,7 +57548,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A340" s="1" t="s">
         <v>4869</v>
       </c>
@@ -57590,7 +57592,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" s="1" t="s">
         <v>4909</v>
       </c>
@@ -57623,7 +57625,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" s="1" t="s">
         <v>4927</v>
       </c>
@@ -57634,7 +57636,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="348" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" s="1" t="s">
         <v>4941</v>
       </c>
@@ -57645,7 +57647,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="349" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A349" s="1" t="s">
         <v>4947</v>
       </c>
@@ -57656,7 +57658,7 @@
         <v>6222</v>
       </c>
     </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" s="1" t="s">
         <v>4949</v>
       </c>
@@ -57667,7 +57669,7 @@
         <v>6226</v>
       </c>
     </row>
-    <row r="351" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" s="1" t="s">
         <v>4965</v>
       </c>
@@ -57678,7 +57680,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="352" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A352" s="1" t="s">
         <v>5007</v>
       </c>
@@ -57689,7 +57691,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="353" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" s="1" t="s">
         <v>5015</v>
       </c>
@@ -57700,7 +57702,7 @@
         <v>6235</v>
       </c>
     </row>
-    <row r="354" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A354" s="1" t="s">
         <v>5033</v>
       </c>
@@ -57711,7 +57713,7 @@
         <v>6229</v>
       </c>
     </row>
-    <row r="355" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A355" s="1" t="s">
         <v>5041</v>
       </c>
@@ -57722,7 +57724,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="356" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A356" s="1" t="s">
         <v>5051</v>
       </c>
@@ -57733,7 +57735,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A357" s="1" t="s">
         <v>5061</v>
       </c>
@@ -57744,7 +57746,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="358" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" s="1" t="s">
         <v>5063</v>
       </c>
@@ -57755,7 +57757,7 @@
         <v>6237</v>
       </c>
     </row>
-    <row r="359" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A359" s="1" t="s">
         <v>5067</v>
       </c>
@@ -57766,7 +57768,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="360" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" s="1" t="s">
         <v>5107</v>
       </c>
@@ -57777,7 +57779,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="361" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A361" s="1" t="s">
         <v>5113</v>
       </c>
@@ -57788,7 +57790,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="362" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A362" s="1" t="s">
         <v>5115</v>
       </c>
@@ -57821,7 +57823,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="365" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" s="1" t="s">
         <v>5167</v>
       </c>
@@ -57832,7 +57834,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="366" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A366" s="1" t="s">
         <v>5191</v>
       </c>
@@ -57854,7 +57856,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="368" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A368" s="1" t="s">
         <v>5209</v>
       </c>
@@ -57887,7 +57889,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="371" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A371" s="1" t="s">
         <v>5233</v>
       </c>
@@ -57898,7 +57900,7 @@
         <v>6210</v>
       </c>
     </row>
-    <row r="372" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A372" s="1" t="s">
         <v>5239</v>
       </c>
@@ -57920,7 +57922,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="374" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A374" s="1" t="s">
         <v>5267</v>
       </c>
@@ -57931,7 +57933,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A375" s="1" t="s">
         <v>5269</v>
       </c>
@@ -57953,7 +57955,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="377" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A377" s="1" t="s">
         <v>5295</v>
       </c>
@@ -57975,7 +57977,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="379" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A379" s="1" t="s">
         <v>5319</v>
       </c>
@@ -57986,7 +57988,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="380" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A380" s="1" t="s">
         <v>5323</v>
       </c>
@@ -58019,7 +58021,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="383" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A383" s="1" t="s">
         <v>5355</v>
       </c>
@@ -58030,7 +58032,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A384" s="1" t="s">
         <v>5359</v>
       </c>
@@ -58052,7 +58054,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="386" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A386" s="1" t="s">
         <v>5367</v>
       </c>
@@ -58063,7 +58065,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="387" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A387" s="1" t="s">
         <v>5395</v>
       </c>
@@ -58074,7 +58076,7 @@
         <v>6224</v>
       </c>
     </row>
-    <row r="388" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A388" s="1" t="s">
         <v>5405</v>
       </c>
@@ -58085,7 +58087,7 @@
         <v>6207</v>
       </c>
     </row>
-    <row r="389" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A389" s="1" t="s">
         <v>5439</v>
       </c>
@@ -58096,7 +58098,7 @@
         <v>6213</v>
       </c>
     </row>
-    <row r="390" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A390" s="1" t="s">
         <v>5443</v>
       </c>
@@ -58118,7 +58120,7 @@
         <v>6205</v>
       </c>
     </row>
-    <row r="392" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A392" s="1" t="s">
         <v>5477</v>
       </c>
@@ -58129,7 +58131,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="393" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A393" s="1" t="s">
         <v>5481</v>
       </c>
@@ -58140,7 +58142,7 @@
         <v>6212</v>
       </c>
     </row>
-    <row r="394" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A394" s="1" t="s">
         <v>5519</v>
       </c>
@@ -58151,7 +58153,7 @@
         <v>6226</v>
       </c>
     </row>
-    <row r="395" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A395" s="1" t="s">
         <v>5537</v>
       </c>
@@ -58162,7 +58164,7 @@
         <v>6232</v>
       </c>
     </row>
-    <row r="396" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A396" s="1" t="s">
         <v>5555</v>
       </c>
@@ -58173,7 +58175,7 @@
         <v>6216</v>
       </c>
     </row>
-    <row r="397" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A397" s="1" t="s">
         <v>5561</v>
       </c>
@@ -58184,7 +58186,7 @@
         <v>6238</v>
       </c>
     </row>
-    <row r="398" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A398" s="1" t="s">
         <v>5575</v>
       </c>
@@ -58195,7 +58197,7 @@
         <v>6211</v>
       </c>
     </row>
-    <row r="399" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A399" s="1" t="s">
         <v>5583</v>
       </c>
@@ -58206,7 +58208,7 @@
         <v>6231</v>
       </c>
     </row>
-    <row r="400" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A400" s="1" t="s">
         <v>5585</v>
       </c>
@@ -58217,7 +58219,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="401" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A401" s="1" t="s">
         <v>5601</v>
       </c>
@@ -58228,7 +58230,7 @@
         <v>6209</v>
       </c>
     </row>
-    <row r="402" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A402" s="1" t="s">
         <v>5623</v>
       </c>
@@ -58239,7 +58241,7 @@
         <v>6206</v>
       </c>
     </row>
-    <row r="403" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A403" s="1" t="s">
         <v>5649</v>
       </c>
@@ -58250,7 +58252,7 @@
         <v>6232</v>
       </c>
     </row>
-    <row r="404" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A404" s="1" t="s">
         <v>5651</v>
       </c>
@@ -58261,7 +58263,7 @@
         <v>6231</v>
       </c>
     </row>
-    <row r="405" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A405" s="1" t="s">
         <v>5681</v>
       </c>
@@ -58272,7 +58274,7 @@
         <v>6223</v>
       </c>
     </row>
-    <row r="406" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A406" s="1" t="s">
         <v>5687</v>
       </c>
@@ -58283,7 +58285,7 @@
         <v>6227</v>
       </c>
     </row>
-    <row r="407" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A407" s="1" t="s">
         <v>5713</v>
       </c>
@@ -58294,7 +58296,7 @@
         <v>6229</v>
       </c>
     </row>
-    <row r="408" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A408" s="1" t="s">
         <v>5721</v>
       </c>
@@ -58306,6 +58308,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C408" xr:uid="{2081DE18-20BE-4B1B-93EE-F628AB19DCC6}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Polar grp: [N+]([O-])"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove Book1.xlsx and add Used_SMILES.xlsx with updated data
</commit_message>
<xml_diff>
--- a/valid_unique_smiles_28_02_2025.xlsx
+++ b/valid_unique_smiles_28_02_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Computer\Meh!!!!!!!\workspace\VIT_LAB\SingletFission_ML\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2A18FD-5918-42F1-9BD0-40B5E5F8777A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301634E2-8FEB-4B7B-A23F-D68A7027A581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="889" firstSheet="2" activeTab="4" xr2:uid="{9748B68E-534E-4D07-B84B-E3A578C6F34D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="889" activeTab="7" xr2:uid="{9748B68E-534E-4D07-B84B-E3A578C6F34D}"/>
   </bookViews>
   <sheets>
     <sheet name="valid_unique_smiles_28_02_2025" sheetId="1" r:id="rId1"/>
@@ -18902,7 +18902,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -19082,6 +19082,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -19243,7 +19249,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -19251,6 +19257,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -54095,13 +54105,13 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="3" t="s">
         <v>6205</v>
       </c>
     </row>
@@ -58461,13 +58471,13 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="3" t="s">
         <v>6190</v>
       </c>
     </row>
@@ -67795,13 +67805,13 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="3" t="s">
         <v>6161</v>
       </c>
     </row>
@@ -70383,13 +70393,13 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="3" t="s">
         <v>6151</v>
       </c>
     </row>
@@ -79769,13 +79779,13 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>448</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="3" t="s">
         <v>6141</v>
       </c>
     </row>
@@ -80861,13 +80871,13 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="3" t="s">
         <v>6134</v>
       </c>
     </row>
@@ -86023,13 +86033,13 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="3" t="s">
         <v>4221</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>4222</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="3" t="s">
         <v>6131</v>
       </c>
     </row>

</xml_diff>